<commit_message>
Problemas con dashboard de docentes y productos educativos
</commit_message>
<xml_diff>
--- a/backend/app/static/plantilla_participantes.xlsx
+++ b/backend/app/static/plantilla_participantes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\Music\lania-certificaciones\backend\app\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{845C86D6-7589-4E34-87B4-EC07F361F2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E33A480F-241E-420E-85B9-3CB8432CEF0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D7818232-5D5C-47DA-B3F1-97B16DB6E749}"/>
   </bookViews>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>full_name</t>
-  </si>
-  <si>
     <t>telefono</t>
   </si>
   <si>
@@ -62,16 +59,19 @@
     <t>para poder subirlos en el sistema</t>
   </si>
   <si>
-    <t>personal_email</t>
-  </si>
-  <si>
     <t>Estos datos no se debe de borrar</t>
   </si>
   <si>
     <t>ni mover de celda</t>
   </si>
   <si>
-    <t>institutional_email</t>
+    <t>nombre_completo</t>
+  </si>
+  <si>
+    <t>email_personal</t>
+  </si>
+  <si>
+    <t>email_institucional</t>
   </si>
 </sst>
 </file>
@@ -559,33 +559,33 @@
   <sheetData>
     <row r="1" spans="2:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="E2" s="5">
         <v>2831054849</v>
@@ -594,7 +594,7 @@
         <v>2831054849</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="18" x14ac:dyDescent="0.35">
@@ -606,12 +606,12 @@
     </row>
     <row r="8" spans="2:8" ht="23.4" x14ac:dyDescent="0.45">
       <c r="D8" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="23.4" x14ac:dyDescent="0.45">
       <c r="D10" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resolucion con el backend
</commit_message>
<xml_diff>
--- a/backend/app/static/plantilla_participantes.xlsx
+++ b/backend/app/static/plantilla_participantes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\Music\lania-certificaciones\backend\app\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E33A480F-241E-420E-85B9-3CB8432CEF0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D283D312-29E1-45A7-839D-2542598BA887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D7818232-5D5C-47DA-B3F1-97B16DB6E749}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>telefono</t>
   </si>
@@ -50,12 +50,6 @@
     <t xml:space="preserve">Sergio Cervantes Guatemala </t>
   </si>
   <si>
-    <t>sergio@lania.edu.mx</t>
-  </si>
-  <si>
-    <t>sergiocervantes@gmail.com</t>
-  </si>
-  <si>
     <t>para poder subirlos en el sistema</t>
   </si>
   <si>
@@ -72,6 +66,15 @@
   </si>
   <si>
     <t>email_institucional</t>
+  </si>
+  <si>
+    <t>Juan Perez Gomez</t>
+  </si>
+  <si>
+    <t>sergiocervantesguatemala@gmail.com</t>
+  </si>
+  <si>
+    <t>meleciomendoza00@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -559,13 +562,13 @@
   <sheetData>
     <row r="1" spans="2:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
@@ -574,7 +577,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
@@ -582,10 +585,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E2" s="5">
         <v>2831054849</v>
@@ -594,7 +597,24 @@
         <v>2831054849</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>2831153752</v>
+      </c>
+      <c r="F3">
+        <v>2831153752</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="18" x14ac:dyDescent="0.35">
@@ -611,15 +631,17 @@
     </row>
     <row r="10" spans="2:8" ht="23.4" x14ac:dyDescent="0.45">
       <c r="D10" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{85DE53FA-E363-4122-9D40-7012CE165CA3}"/>
-    <hyperlink ref="C2" r:id="rId2" xr:uid="{C36170B0-F434-4B77-88AA-9B0EB498F5B1}"/>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{C36170B0-F434-4B77-88AA-9B0EB498F5B1}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{7E69275B-9D1D-47FC-9CED-2DF47AB023ED}"/>
+    <hyperlink ref="D2" r:id="rId3" xr:uid="{39FDB3BC-EC1F-4ACF-B541-314F54A93B53}"/>
+    <hyperlink ref="D3" r:id="rId4" xr:uid="{07034DBF-9206-4A6A-BD5A-26562E8591B4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>